<commit_message>
version 53 - Improve Knowledge type classification and test recall method for validation
</commit_message>
<xml_diff>
--- a/FastAPI_AI_Service/app/data/NenThom_data/Product_Catalogs/Tests/Results/Result_Test_Accesories_product_only.xlsx
+++ b/FastAPI_AI_Service/app/data/NenThom_data/Product_Catalogs/Tests/Results/Result_Test_Accesories_product_only.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,7 +437,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.58</v>
+        <v>12.81</v>
       </c>
     </row>
     <row r="6">
@@ -477,7 +477,27 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19.3</v>
+        <v>17.43</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Avg_Judge_Latency</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6.99</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P95_Judge_Latency</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>10.41</v>
       </c>
     </row>
   </sheetData>
@@ -491,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -530,6 +550,11 @@
           <t>Response Time</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Judge Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -544,19 +569,21 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Luận điểm: Việc sử dụng kẹp/che tắt nến chuyên dụng có tay cầm dài loại bỏ hoàn toàn cả nguy cơ hỏa hoạn chính và ô nhiễm mùi do thổi tắt bằng miệng.
-Cơ sở lập luận
-- Khoảng cách và bảo vệ vật lý  
-  - Tay cầm dạng que thẳng rất dài với tay nắm công thái học tối đa hóa khoảng cách giữa người dùng và ngọn lửa, giữ chặt và chống trượt, đồng thời bảo vệ ngón tay khỏi phơi nhiễm nhiệt nặng khi với sâu vào nến cột cao.  
-- Ngăn chặn khói và muội than ngay lập tức  
-  - Dụng cụ che tắt cắt đứt oxy tức thì, hoàn toàn loại bỏ mùi khói sau khi đốt và sinh muội than đen, nên không phá hỏng hiệu năng mùi hương còn lại trong phòng.  
-- Loại trừ bắn tung sáp nóng và sự cố do thổi mạnh  
-  - Thay thế hành động thổi mạnh bằng che tắt loại đầu xoay hoàn toàn loại trừ rủi ro bắn ngược sáp lỏng, ngăn sáp nóng bắn lên đồ đạc, vải vóc hoặc lên mặt và da người.  
-  - Hành động thổi còn tạo ra luồng puff kéo dài gây muội than và mùi cháy; che tắt chuyên dụng loại bỏ những tác nhân này.
-- Mục tiêu tổng thể của dụng cụ chăm sóc nến  
-  - Sử dụng kéo và che tắt chuyên dụng cho phép tận hưởng thẩm mỹ và mùi thơm của nến trong khi hoàn toàn loại bỏ rủi ro hỏa hoạn, muội than đen và tai nạn tràn/ bắn sáp.
-Kết luận  
-Kết hợp yếu tố (1) khoảng cách bảo vệ, (2) cắt oxy tức thì để ngăn khói và muội than, và (3) ngăn bắn sáp nóng, dụng cụ che tắt nến tay dài loại trừ triệt để cả nguy cơ hỏa hoạn chính và ô nhiễm mùi phát sinh khi thổi tắt bằng miệng.</t>
+          <t>Structured argument — why a specialized long-handled candle snuffer removes the main fire hazards and odor contamination from blowing out wicks
+Thesis
+- Using a specialized long-handled candle snuffer eliminates the primary hazards and odor contamination that result from blowing out candle wicks.
+Premises
+- Blowing a candle produces a prolonged puff of toxic black soot, an intense burnt smell that ruins the room’s fragrance, and risks splattering liquid wax across surfaces.
+- A snuffer cuts off oxygen instantly, which completely eliminates post-burn smoke smell and black soot generation.
+- A pivoting-head snuffer completely eliminates the risk of messy liquid wax blow-back, preventing hot wax from splattering onto furniture, textiles, or the user’s face and skin.
+- An extra-long straight rod handle with an ergonomic, textured grip maximizes physical distance from the flame, protects fingers from severe heat, prevents slippage, and ensures a steady hand when reaching into deep or tall candle vessels.
+Logical steps
+- Because a snuffer cuts off oxygen instantly, there is no prolonged smoke-producing puff; therefore the source of black soot and the burnt odor is removed at extinguishing.
+- Because the snuffer does not rely on a forceful air puff, it avoids creating any blow-back currents that can splatter hot wax; the pivoting head design further prevents wax blow-back entirely.
+- Because the long handle and textured ergonomic grip keep the user well away from the flame and provide secure control, the risk of accidental contact with hot wax or the flame (burns or igniting nearby materials) is removed.
+- Eliminating both the smoke/soot source and the wax-splatter mechanism removes the two primary pathways by which blowing out a wick creates fire-safety hazards and contaminates room fragrance.
+Conclusion
+- By extinguishing the flame through immediate oxygen cutoff, preventing wax blow-back, and keeping the user safely distant with a secure grip, a specialized long-handled candle snuffer effectively and entirely eliminates the main fire-hazard and odor-contamination problems caused by blowing out candle wicks.</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -569,7 +596,10 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>22.25</v>
+        <v>15.12</v>
+      </c>
+      <c r="H2" t="n">
+        <v>6.06</v>
       </c>
     </row>
     <row r="3">
@@ -585,19 +615,18 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A professional wick trimmer uses a few specific structural features to keep white soy wax pools clean and to promote a controlled, uniform melt pool:
-Structural features and their effects
-- Integrated disc-shaped / flat circular catch tray
-  - Immediately captures clipped, soot-covered carbon tips so they cannot fall back into the wax.
-  - Keeps pristine white soy wax from becoming discolored or contaminated by black debris.
-- Horizontal debris catch basin (disc tray) sized for multi-wick work
-  - Catches clippings from several wicks at once, preventing multiple snips from dropping soot into wide wax pools.
-  - Makes cleanup easy and avoids fishing sticky debris out of the wax.
-- Long reach for cutting deep inside tall containers and precise cutting to the ideal height
-  - Trims wicks down to the recommended quarter-inch height, which prevents oversized or erratic flames.
-  - A properly shortened wick leads to a controlled, uniform wax melt pool and steadier burn, reducing soot production and slowing wax consumption.
-Net result
-- The combined design both physically prevents soot from contaminating the wax (catch tray/basin) and ensures optimal wick length for a stable flame and even melt pool, preserving the look and burn performance of white soy candles.</t>
+          <t>How the trimmer’s structure protects white soy wax pools and controls the melt pool
+- Precise cutting reach
+  - A specialized trimmer is shaped to cut wicks deep inside tall containers down to the ideal quarter-inch height.
+  - This prevents overgrown braided cotton wicks that cause erratic, oversized flames and uneven melt pools.
+- Integrated horizontal catch basin / flat circular tray
+  - A disc-shaped catching basin directly beneath the cutting blades immediately captures the snipped carbon tips.
+  - For multi-wick candles, the tray catches clippings from multiple wicks at once, preventing debris from falling into wide wax pools.
+- Direct effects on wax cleanliness and burn behavior
+  - By catching soot-covered carbon clippings before they drop, the trimmer prevents blackened debris from contaminating or discoloring pristine white soy wax.
+  - Trimming to the proper height and removing clippings ensures a controlled, uniform wax melt pool, reduces soot deposits, and regulates wax consumption — helping extend total burn hours.
+- User experience benefit
+  - The built-in catch tray makes candle care cleaner and more satisfying by eliminating the need to fish dirty debris out of sticky wax.</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -610,7 +639,10 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>10.32</v>
+        <v>9.77</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5.96</v>
       </c>
     </row>
     <row r="4">
@@ -626,17 +658,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>How it works (thermodynamic principle)
-- The candle flame heats the air above it, producing rising hot thermal air currents.
-- Those upward currents strike the angled blades of a delicate, multi-blade metal turbine and push against them.
-- The angled blades convert the upward airflow into continuous rotation, so the carousel spins automatically via thermodynamics — without any electrical power.
-Design strategy to create dynamic moving shadows
-- Angled multi-blade metal turbine: blade angle and multiple blades ensure a steady, smooth spin from the rising air.
-- Integrated circular metal well: holds a standard tealight firmly in place so the heat source doesn’t shift, producing consistent rising air currents for stable rotation.
-- Dangling metallic charms: mounted on the rotating carousel, they spin gracefully and cast rhythmic, dancing shadows across walls and mirrors.
-- High-shine reflective plating on the turbine: bounces the candle’s firelight upward and outward, amplifying and maximizing the shifting patterns of light and shadow across the ceiling and room.
-Resulting effect
-- The combination of steady convective updraft, rotating blades, reflective surfaces, and spinning charms produces continuous, dynamic moving shadows and a whimsical, cozy visual atmosphere — all driven solely by the candle’s heat.</t>
+          <t>Summary
+A heat-powered candle carousel uses the candle’s hot air alone to spin a small turbine and produce moving shadows — no electricity required.
+Technical design strategy and thermodynamic principles
+- Heat-driven rotation  
+  - The candle flame creates rising hot thermal air currents.  
+  - Those updrafts strike the angled blades of a delicate multi-blade metal turbine mounted at the top, pushing the blades and converting the thermal updraft into smooth rotational motion.
+- Stable and directed airflow  
+  - An integrated circular metal well holds a standard tealight firmly in place so the heat source doesn’t shift, ensuring steady, consistent rising air currents that keep the turbine turning.
+- Shadow and light optimization  
+  - Dangling metallic charms attached to the rotating assembly spin as the turbine turns, casting rhythmic, dancing shadows across walls and mirrors.  
+  - A high-shine reflective plating on the metal turbine bounces the candle’s firelight upward and outward, maximizing shifting patterns of light and shadow across the room.
+- Resulting effect and user experience  
+  - The combination of thermally driven rotation, moving charms, and reflective surfaces produces dynamic, moving shadows and a whimsical, enchanting, cozy, and calming atmosphere.</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -649,7 +683,10 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>13.88</v>
+        <v>13.4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.18</v>
       </c>
     </row>
     <row r="5">
@@ -678,7 +715,10 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>15.1</v>
+        <v>8.27</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.64</v>
       </c>
     </row>
     <row r="6">
@@ -694,26 +734,33 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Why include cross-cut pine wood tray discs in luxury candle gift sets and lifestyle flat-lay photography
+          <t>Here’s a clear, usable case you can make to justify adding cross-cut pine wood tray discs to luxury candle gift sets and lifestyle flat-lay photography.
 Utility benefits
-- Acts as a heat-resistant protective layer for tabletops and packaging—prevents heat damage, wax drips, and soot deposits.
-- Provides stable bases and step-risers for candles, small jars, mugs, or planters—reduces accidental spills and surface marks.
-- Multi-use: suitable as coasters, decorative centerpieces, and display risers for events or retail setups.
-Aesthetic benefits
-- Unique organic growth rings and textured bark edges create a warm, handcrafted backdrop that visually elevates luxury candles and makes them stand out in flat-lays.
-- Conveys a rustic, cozy, and grounded mood that complements minimalist or natural-branding aesthetics.
-- Year‑round versatility: works for autumn/winter cozy scenes, rustic summer weddings, and everyday lifestyle photography.
-Relevant product details (why they matter)
-- Material: 100% premium natural pine wood — authentic, tactile feel that reads as high-quality and handmade.
-- Finish: smoothly sanded faces with preserved rough bark trim — clean surface for display while keeping organic texture.
-- Thickness: typically 1.0–1.5 cm — thin enough to include in gift sets, sturdy enough to protect surfaces.
-- Shape: organic circular/oval slices — looks natural and photographic without being rigidly uniform.
-How to use them effectively
-- Place a disc under each candle inside a gift box to protect the box and add a premium unboxing moment.
-- Use stacked discs as risers in flat-lays to create depth and highlight a hero candle.
-- Pair with simple match slide-boxes or elegant metal trays to complete a curated self-care or gift set presentation.
-Bottom line
-Cross-cut pine wood discs deliver both practical protection and an immediate visual upgrade—adding tangible safety benefits while reinforcing a handcrafted, luxury brand story.</t>
+- Heat protection and stability  
+  - Heat-resistant discs protect tabletops and packaging from hot candle jars and melted wax.  
+  - Smoothly sanded faces give stable, safe surfaces for candles while the rough bark edge stays intact for grip and character.
+- Safety and care advantages  
+  - Using high-quality accessories like these helps prevent soot deposits and accidental wax damage, supporting safer candle use and presentation.
+- Functional display element  
+  - Serve as practical step-risers and protective bases for jars, making multi-layered packaging and tiered product displays easy and secure.
+- Relevant specifications (helpful for sourcing/production)  
+  - Material: 100% real premium pine wood.  
+  - Thickness: typically 1 cm to 1.5 cm for stable support.  
+  - Shape: organic circular or slightly oval slices.
+Aesthetic and branding benefits
+- Photogenic, luxury-ready backdrop  
+  - Unique growth rings and textured bark edges create a warm, handcrafted visual riser that makes luxury candles and small objects stand out in lifestyle flat-lays.
+- Strong mood and storytelling signals  
+  - Conveys rustic, organic, cozy, minimalist, and earthy vibes — ideal for brands emphasizing natural, artisanal, or slow-living values.
+- Perceived value and versatility  
+  - Seen by customers and small-business sellers as charming and premium; adding a natural wood disc elevates gift-set presentation and can make product imagery feel more intentional and boutique.
+Practical use cases to highlight to buyers
+- As a protective coaster inside gift sets to prevent heat or wax transfer to packaging.  
+- As a visual riser in flat-lay photography and product shots to add depth and focus.  
+- As a tabletop centerpiece or display base in retail photos and at events to reinforce a handmade, natural brand story.  
+- As a multipurpose accessory in bundles (candle + snuffer/trimmer + wood disc) to communicate completeness and care.
+Closing summary
+Cross-cut pine wood tray discs deliver both measurable utility (heat protection, safer candle use, stable displays) and strong aesthetic lift (photogenic texture, warm handcrafted cues, elevated perceived value). They are a small, low-effort addition that strengthens product safety, photography, and the overall luxury presentation of your candle gift sets.</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -726,7 +773,10 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>16.98</v>
+        <v>14.99</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5.31</v>
       </c>
     </row>
     <row r="7">
@@ -742,19 +792,21 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Product configuration
-- Premium textured rose‑gold (or amber) glass candle vessel with a deeply textured pattern.
-- Polished yellow‑gold candle carousel with **integrated tealight well** and **delicate hanging ornaments**.
-- Pair with a premium holiday candle such as Voluspa’s "Gilt Pomander &amp; Hinoki" for the fragrance/mood layer.
-Why this satisfies the brief
-- The deeply textured rose‑gold/amber vessel becomes an artistic statement that catches and scatters ambient light, giving a luxurious, decorative glow even when the flame is low.
-- The polished yellow‑gold carousel supplies the kinetic element: its brilliant reflective plating and moving, hanging ornaments create a festive, conversation‑sparking display centered around the tealight.
-- The fragrance/mood layer (e.g., "Gilt Pomander &amp; Hinoki") brings a dreamy, magical, mesmerizing, luxurious, warm, festive, and therapeutic atmosphere — exactly the winter holiday ritual mood the consumer seeks.
-This pairing delivers a high‑end, therapeutic holiday accent piece by combining tactile visual luxury, gentle motion, and an immersive seasonal scent.</t>
+          <t>Recommended configuration
+- Premium textured rose‑gold or amber glass candle vessel  
+  - Deeply textured pattern that turns the container into an artistic statement and catches ambient room light — adds a luxe, restful visual focus for a ritual.
+- Polished yellow‑gold candle carousel with integrated tealight well and delicate hanging ornaments  
+  - Kinetic moving elements create a festive, conversational centerpiece and gentle motion that enhances ritual presence.
+- Scent choice: Voluspa "Gilt Pomander &amp; Hinoki" (holiday fragrance)  
+  - Mood profile: dreamy, magical, mesmerizing, luxurious, warm, festive, and **therapeutic** — aligns directly with a high‑end winter holiday ritual.
+Why this satisfies the target mood
+- The textured glass provides the premium, calming visual and tactile quality expected of a therapeutic accent piece.  
+- The gold carousel supplies kinetic motion and holiday sparkle, turning the setup into a moving ritual centerpiece.  
+- The chosen fragrance profile adds warmth, luxury, and a therapeutic atmosphere, completing a cohesive winter holiday ritual experience.</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -763,7 +815,10 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>17.51</v>
+        <v>11.36</v>
+      </c>
+      <c r="H7" t="n">
+        <v>7.08</v>
       </c>
     </row>
     <row r="8">
@@ -779,17 +834,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Technical packaging elements
-- Heavy-duty slider matchbox housing — a sturdy slide-box design that holds elongated sticks securely for easy single-handed access.  
-- Honeycomb-textured friction strike pad running along the side panel — engineered for smooth, reliable, wind-resistant ignition even after long periods of storage.  
-- Elongated natural wood splints stored in the slider — designed for clean, steady strikes and extra-long burn time.  
-- Match tips finished with high-quality, clean-burning safety chemicals — formulated for consistent ignition when struck against the friction pad.
-Physical safety advantages over standard disposable lighters
-- Extra-long burn time from the elongated wooden sticks lets you light deep wax wicks without bringing your fingers close to the flame, reducing burn risk.  
-- Clean-burning tips and even-burning wood splints provide steady, reliable ignition (less need for repeated attempts that expose hands to flame).  
-- Honeycomb strike pad + stable tip chemistry = smooth, wind-resistant ignition and dependable performance after storage, so you’re less likely to fumble when lighting.  
-- Natural wood splints offer structural stiffness for controlled handling into tall glass jars, making them safer for deep-wick candles than short, handheld disposable lighters.  
-Overall, the combination of the slider packaging, textured strike surface, elongated wood sticks, and clean-burning tip chemistry delivers more controlled, reliable, and safer ignition for deep jar candles than standard disposable plastic lighters.</t>
+          <t>### Artisanal Minimalism Candle Matchbox — Technical packaging elements
+- Packaging: heavy-duty slider matchbox with a honeycomb-textured friction strike pad running along the side panel.
+- Match construction: elongated natural aspen wood splints tipped with high-quality, clean-burning (sulfur-free) safety chemicals.
+- Form factor: extra-long wooden sticks sized for reaching into deep glass jars and multi-wick candles.
+- Protective packaging: robust slider housing keeps matches secure and limits accidental friction/ignition during storage and handling.
+### Physical safety advantages over standard disposable lighters
+- Greater reach: elongated sticks keep fingers well away from flames when lighting deep-wick or tall jar candles, reducing burn risk.
+- Predictable, clean burn: natural wood splints and clean-burning tips provide steady, controlled ignition without the irregular flame behavior sometimes found with cheap lighters.
+- Reliable ignition over time: the honeycomb-textured strike pad plus stable safety chemicals ensure smooth, wind-resistant lighting even after long storage.
+- Safer handling and storage: the heavy-duty slider box protects match heads and limits unintended strikes, lowering accidental-ignition risk compared with exposed lighter mechanisms.
+- Structural consistency: natural wood splints burn evenly and maintain stiffness, giving predictable performance when reaching into narrow or deep containers.</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -802,7 +857,10 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>19.15</v>
+        <v>11.17</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6.06</v>
       </c>
     </row>
     <row r="9">
@@ -818,24 +876,25 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Candle holder (unscented white bear under glass dome)
-- Consumer perception:
-  - Cute, charming, whimsical, and heartwarming.
-  - Seen as a handcrafted minimalist decorative object.
-  - Valued for its aesthetic and ability to create a cozy atmosphere even when unlit.
-- Primary use-case:
-  - Decorative display (bedroom, desk, living room, nursery, photo props, shelf).
-  - Gift item for aesthetics/collecting rather than for fragrance or aromatherapy.
-Dalat Gift (scented candle + travel perfume set)
-- Consumer perception:
-  - Nostalgic, relaxing, artistic, and high-end/ thoughtfully curated.
-  - Appreciated for its evocative pine/moss/lemon/amber scent that captures a misty, highland mood.
-  - Loved for the combination of a home candle plus a personal fragrance spray and attractive rustic packaging.
-- Primary use-case:
-  - Functional aromatherapy and personal fragrance: scenting rooms, creating a cozy/grounding atmosphere, and carrying a travel perfume.
-  - Gift set for calming self-care, birthdays, travel souvenirs, or creating a curated sensory experience.
-Summary contrast (one line)
-- The bear candle is primarily an aesthetic decorative object and collectible that adds visual coziness; the Dalat Gift is a multisensory, functional aromatherapy gift set designed to scent spaces and support relaxation and personal fragrance use.</t>
+          <t>Here’s a clear contrast between the two products.
+Candle holder (white bear under glass)
+- Consumer perception
+  - Cute, charming, minimalist, handcrafted and whimsical.
+  - Seen as a decorative, heartwarming object that creates a cozy atmosphere even unlit.
+  - Popular as a gift for its aesthetic and collectible appeal.
+- Ultimate primary use-case
+  - Decorative display piece (bedroom, desk, living room, nursery, photography prop, shelf).
+  - Bought mainly for visual/aesthetic value rather than fragrance or aromatherapy.
+Dalat Gift (scented candle + travel perfume gift set)
+- Consumer perception
+  - Nostalgic, relaxing, artistic, and high-end in presentation.
+  - Evokes pine forests and misty highland moods; praised for sensory curation and thoughtful unboxing.
+- Ultimate primary use-case
+  - Functional aromatherapy and multi-sensory gift: creates a pine/woody indoor atmosphere and offers a companion travel perfume.
+  - Suited for therapeutic self-care, calming workspaces, souvenirs, and gifting to those who appreciate scent-driven experiences.
+Bottom line
+- The bear candle under glass is primarily an aesthetic object valued for looks and atmosphere without needing to be lit.
+- The Dalat Gift is a purposeful fragrance experience designed to be used—burned and worn—to evoke mood, nostalgia, and relaxation.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -848,7 +907,10 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>11.09</v>
+        <v>9.06</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8.75</v>
       </c>
     </row>
     <row r="10">
@@ -864,20 +926,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>How each finish changes the decor statement
-- Polished Chrome Silver  
-  - Clean, contemporary look that fits modern interiors.  
-  - Resists fingerprint smudges better than highly polished gold, so it reads sleek and understated in high‑traffic spaces.
-- Iridescent Rainbow  
-  - Adds an eye‑catching, multi‑tone metallic pop that breaks up monochrome or Nordic styling.  
-  - Reflects shifting colors as lighting changes, creating a dynamic, playful accent.
-- Metallic Gold (e.g., luxury rose‑gold family)  
-  - Conveys a more luxurious, personalized feel—turning a routine candle ritual into a stylish self‑care detail that suits classic or elevated interiors.
-Why the furniture protection stays the same
-- The tray’s base material is food‑grade stainless steel, which provides superior density, premium weight, and strong rust resistance so the surface remains stain‑free even with candle oils.  
-- Smooth, rounded edges ensure safe handling without sharp corners.
-Bottom line
-- Finish choice alters only the visual and stylistic statement (modern, playful, or luxurious), while the stainless steel construction and rounded design preserve identical protection and functionality.</t>
+          <t>Brief answer
+Different finishes change the visual and emotional impact of the tray while the tray’s construction and safety features keep furniture protection identical.
+Brilliant Yellow Gold
+- Gives a metallic, luxury-style statement that turns everyday ritual into a personalized, stylish moment (metallic finishes are linked to a heightened luxury feel).
+- May show more fingerprint smudging compared with polished chrome.
+- Offers the same furniture protection as the other finishes because the tray’s material and design remain unchanged.
+Polished Chrome Silver
+- Presents a clean, contemporary look that suits modern interiors.
+- Resists fingerprint smudges better than highly polished gold, keeping the surface looking cleaner with heavy use.
+- Maintains identical protection for furniture through the same underlying construction.
+Iridescent Rainbow
+- Adds an eye-catching, multi-tone metallic pop that breaks up monochromatic spaces and shifts color with changing light—good for Nordic or minimalist settings that need a visual accent.
+- Delivers the same protective performance as other finishes.
+Why protection stays the same
+- The tray uses food‑grade stainless steel with superior density, premium weight, rust resistance, and stain resistance, so it protects furniture equally well regardless of finish.
+- Smooth, rounded edges ensure safe handling and preserve the tray’s protective function while keeping a sleek aesthetic.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -890,7 +954,10 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>12.91</v>
+        <v>17.33</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4.85</v>
       </c>
     </row>
     <row r="11">
@@ -906,14 +973,15 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Short answer
-Sulfur-free tips prevent any stray sulfur or harsh chemical odor at ignition, so the candle’s true fragrance is not masked when you light it.
-Why that matters — technical points
-- Sulfur-free safety chemicals do not release the rotten-egg/sulfur smell that appears when sulfur-tipped matches are struck, so the very first scent you perceive is the candle’s essential-oil aroma, not a combustion off-note.  
-- Clean-burning tip formulations eliminate the pungent, harsh chemical odor typical of cheap lighters, preserving the candle’s pure initial scent throw.  
-- Using eco-friendly natural wood splints with clean-burning tips supports an even, high-end lighting experience that complements luxury aromatherapy rituals without introducing unwanted odors.
-Bottom line
-A sulfur-free tip keeps the ignition step odor-neutral, allowing the candle’s intended fragrance profile to come through clearly from the moment it’s lit.</t>
+          <t>Key technical reasons a sulfur-free match tip preserves a luxury candle’s true scent throw
+- Prevents sulfur odors that mask fragrance  
+  Sulfur-containing tips release a harsh, rotten-egg sulfur odor when struck. That odor can overpower or alter the candle’s essential-oil aroma at the moment of ignition.
+- Ensures a clean initial scent impression  
+  Sulfur-free safety chemicals burn cleanly and do not produce the pungent, chemical smell typical of cheap disposable lighters or sulfur-tipped matches, so the room is filled by the candle’s intended fragrance instead of combustion byproducts.
+- Keeps the match itself effectively unscented  
+  Matches designed as unscented (natural aspen wood with a sulfur-free tip) avoid adding any competing scent notes, helping the candle’s top notes come through as intended.
+- Supports consistent, minimal-contamination burning  
+  Natural wood splints burn evenly and with good structural stiffness, contributing to predictable ignition without introducing extra odors or residues that could interfere with the candle’s aroma.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -926,7 +994,10 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>8.380000000000001</v>
+        <v>10.33</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5.42</v>
       </c>
     </row>
     <row r="12">
@@ -942,14 +1013,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>### Structural role of the smooth rounded metal ball feet
-- They raise the tray slightly off the tabletop, preventing scratches on delicate furniture surfaces.  
-- They create an insulating air gap under the tray that minimizes thermal transfer.  
-- Paired with the polished gold mirror vanity tray’s containment of diffusers and cosmetics, the elevation helps preserve the underlying paint or veneer finish.</t>
+          <t>Role of the smooth rounded metal ball feet
+- Slight elevation of the tray off the tabletop, preventing scratches on delicate furniture surfaces.  
+- Creation of an insulating air gap that minimizes thermal transfer to the surface underneath.
+These features help protect the underlying tabletop when the tray holds cosmetics and oil diffusers.</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -958,7 +1029,10 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>10.91</v>
+        <v>13.49</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5.98</v>
       </c>
     </row>
     <row r="13">
@@ -974,18 +1048,18 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>How an overgrown, untrimmed wick creates black soot
-- An overlong wick produces a larger, hotter flame and an inconsistent burn rate.  
-- That condition lets the wick draw up excess liquid wax and oxygen at the same time, promoting incomplete combustion.  
-- Incomplete combustion forms soot (carbonized particles) and visible black smoke.  
-- Split or carbonized wick tips act as additional soot sources, which deposit as black rings on glass walls and release airborne soot into the indoor environment.
-How a professional wick trimmer removes the hazard
-- Precisely sets wick length: trimming to a short, controlled height (documents note trimming to approximately **3 mm** after each use, and an ideal quarter-inch height for deep cuts in tall containers) keeps flame size and burn rate consistent.  
-- Removes carbonized/split tips: cutting away the charred ends prevents those sites from producing excess soot.  
-- Built-in debris control: a professional trimmer’s integrated disc-shaped catching basin traps carbon debris so it cannot fall back into or contaminate the wax pool.  
-- Reaches deep wicks safely: the tool is designed to cut wicks that sit far down inside tall jars, ensuring the correct wick length even in deep containers.
-Net effect
-- Controlled flame and cleaner combustion reduce or eliminate black smoke and soot deposits on glass and in the air, keeping the wax pool and jar interior cleaner and improving indoor air quality.</t>
+          <t>How an overgrown, untrimmed wick produces black soot
+- An overgrown wick produces a larger, uncontrolled flame that changes the burn dynamics.
+- That larger flame allows the wick to draw up excess wax and oxygen at the same time, which promotes incomplete combustion.
+- Incomplete combustion creates soot-filled black smoke and airborne soot particles that deposit as black rings on glass and as general residue.
+- Carbonized and split wick ends act as additional soot sources; if left untrimmed they generate excess soot and cause black smoke rings on jar walls.
+- Over time, this soot release negatively affects indoor air cleanliness by increasing airborne soot particles.
+How a professional wick trimmer structurally eliminates the hazard
+- Precise cutting: a trimmer is designed to accurately cut the wick to a controlled ideal height (documents reference trimming to approximately **3 mm** after each use and specialized trimmers that cut down to an **ideal quarter-inch** height), which limits flame size and stabilizes burn rate.
+- Debris capture: many professional trimmers include an integrated disc-shaped catching basin to trap the carbonized wick clippings and prevent them from falling into and contaminating the wax pool.
+- Deactivates soot sources: by removing carbonized, split wick ends, the trimmer stops the formation of excessive soot, preventing black smoke and black smoke rings on glass walls.
+- Promotes complete combustion: keeping the wick clean and trimmed maintains clean, complete combustion of the wax, reducing the release of airborne soot particles and black smoke into the indoor environment.
+Result: regular use of a professional wick trimmer controls flame size, removes carbonized wick material, and captures debris — together these actions prevent soot generation, keep glass and wax clean, and protect indoor air quality.</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -998,7 +1072,10 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>9.779999999999999</v>
+        <v>10.35</v>
+      </c>
+      <c r="H13" t="n">
+        <v>9.31</v>
       </c>
     </row>
     <row r="14">
@@ -1015,18 +1092,18 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>Thermodynamic safety features
-- Integrated metal tealight well sized for standard aluminum or clear-cup tealights — the metal well manages and contains the candle’s heat source in a dedicated pocket.
-- Heat‑responsive precision‑stamped alloy construction and high‑shine plating — materials engineered to tolerate and respond predictably to the thermal flow produced by a burning tealight.
-- Design that uses rising hot air currents to drive the turbine — the carousel channels predictable thermal currents for motion rather than relying on uncontrolled flames or drafts.
+- Heat‑responsive lightweight alloy construction that is engineered to work with rising hot air, directing thermal currents through the multi‑blade turbine rather than letting heat concentrate unpredictably.  
+- An integrated circular metal tealight well that contains the candle and its heat source in a defined metal cup area.  
+- Use of an anti‑rust metal frame plus a mirrored glass base (tray design) that prevents high heat from standard glass candle bottoms from directly transferring to wood, laminate, or marble tabletops, and also catches any hot wax mishaps.
 Mechanical safety features
-- Metal cup holder that locks the tealight into place, preventing it from sliding or tipping if the table is bumped.
-- Sturdy alloy frame and secure base design that hold the candle and spinning parts in a fixed arrangement, reducing the chance of accidental contact with the flame or ornaments.
-- (Where present in related metal candle trays) an anti‑rust metal frame and mirrored glass base that catch hot wax and prevent direct transfer of high heat from candle bottoms to vulnerable tabletops.
-How this compares with open un‑contained candle holders
-- Stability: the carousel’s locking metal well reduces tipping/ sliding risk; open un‑contained holders lack that confined cup and therefore do not physically secure small tealights in the same way.
-- Heat management: the carousel’s metal base and heat‑responsive materials contain and channel thermal energy; open holders (for example, standard glass bottoms) can allow direct heat transfer to the table and are less likely to catch hot wax cleanly.
-- Predictable behavior: the carousel is engineered to use predictable thermal airflow for motion, while open holders do not integrate that controlled thermodynamic design.
-If you need a short checklist to evaluate a specific polished yellow gold carousel’s safety (what to look for), I can provide one.</t>
+- A secure, integrated metal tealight cup holder that locks the small tealight into a metal well so the candle cannot slide or tip if the table is bumped.  
+- Precision‑stamped construction with a curved support rod and a balanced multi‑blade turbine designed for stable, predictable motion as the carousel spins.  
+- Durable plated finishes (polished yellow gold) and anti‑rust metal framing that maintain structural integrity around the heat source.
+How that compares to open un‑contained candle holders
+- The carousel’s locked metal well and cup holder actively prevent sliding or tipping; open, un‑contained holders do not provide that built‑in locking cup.  
+- The mirrored glass base and metal frame reduce direct heat transfer to delicate surfaces and catch wax spills; open setups without such containment allow heat and wax to contact tabletops.  
+- The design channels thermal updrafts to drive the turbine, converting heat into controlled motion rather than leaving heat to disperse unpredictably.
+If you need exact specifications for a specific gold carousel model (dimensions, base materials, or tested heat‑ratings), you should contact admin for detail information.</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1039,7 +1116,10 @@
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>18.02</v>
+        <v>16.69</v>
+      </c>
+      <c r="H14" t="n">
+        <v>7.08</v>
       </c>
     </row>
     <row r="15">
@@ -1055,26 +1135,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>### Gift set identified
-Dalat Gift — Heny Garden
-### Why it fits the request
-- Evokes a chilling, misty pine-forest mood (pine wood, green moss, cedarwood, cold lemon peel, warm amber).
-- Combines organic timber elements and heat-safe wood accessory with both a personal fragrance (travel perfume) and a room fragrance (candle).
-### Structural contents (breakdown)
-- **Packaging**
-  - Sturdy kraft paper gift box filled with paper crinkle shreds.
-- **Scented candle (Đà Lạt)**
-  - Clear glass candle jar with a natural, eco-friendly light **bamboo wooden lid**.
-  - Wax seal emblem on the jar.
-  - Key scent profile: pine wood &amp; moss heart; lemon peel top; dry amber and cedarwood base.
-- **Personal fragrance**
-  - Mountain Tea Eau de Toilette — **10 ml** travel-sized clear glass spray bottle with a sleek black cap.
-- **Organic timber element**
-  - Thick natural **cross-cut pine log coaster** (heat-resistant, rustic timber accent).
-- **Botanical decor / unboxing visuals**
-  - Dried cream hydrangea bouquet accented with bunny tail stems.
-  - Two dehydrated real orange slices.
-If you need this formatted for a product page or a packing checklist, I can produce that next.</t>
+          <t># Gift set: Dalat Gift
+This gift box matches a chilling forest mood and combines organic timber elements with both personal and room fragrances.
+Structural contents and key details
+- Brand: **Heny Garden**
+- Category: Scented Candle &amp; Travel Perfume Gift Set
+- Main scents / Fragrance family / Mood:
+  - Scents: **Pine Wood, Fresh Moss, Lemon Peel, Warm Amber, Cedarwood, Mountain Tea**
+  - Fragrance family: **Earthy Woody / Fresh Aromatic Botanical**
+  - Mood: **Nostalgic, peaceful, misty, grounding, refreshing, cozy**
+- Physical contents:
+  - **"Đà Lạt" scented candle** in a clear glass jar (pine &amp; moss-led scent), topped with a natural **bamboo wooden lid** and accented by a **wax seal emblem**.
+  - **10 ml Mountain Tea eau de toilette** travel spray (clear glass bottle with black cap) — personal fragrance.
+  - **Thick natural cross-cut pine log coaster** (organic timber element / protective base).
+  - **Dried cream hydrangea bouquet** with bunny tail stems — rustic dried-flower accent.
+  - **Two dehydrated real orange slices** — decorative sensory detail.
+  - **Sturdy kraft paper gift box** filled with **paper crinkle shreds** for presentation and protection.
+- Useful specs:
+  - Candle variation labeled **Đà Lạt** (key notes: pine &amp; moss, lemon peel, amber, cedarwood).
+  - Coaster material: **100% natural pine wood**.
+  - Perfume size: **10 ml** travel spray.
+This set offers a cohesive unboxing that recreates a chilly pine-forest atmosphere while combining a home candle (room fragrance), a travel eau de toilette (personal fragrance), and tactile organic timber details.</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1087,7 +1168,10 @@
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>8.470000000000001</v>
+        <v>11.75</v>
+      </c>
+      <c r="H15" t="n">
+        <v>5.83</v>
       </c>
     </row>
     <row r="16">
@@ -1103,21 +1187,21 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Each charm variation—silver snowflakes, standing pine trees, and whimsical reindeer—changes the winter festive atmosphere in ways customers frequently notice:
-Silver snowflakes
-- High-shine silver finish catches and multiplies light from the candle, amplifying a magical, wintry glow.
-- Rotating motion creates mesmerizing, rhythmic movement that customers describe as dreamy and therapeutic.
-- Combined with textured embossed glass, the snowflakes intensify reflections and cast dancing patterns that elevate a table or mantel into a sophisticated focal point.
-Standing holiday pine trees
-- Evoke a classic, traditional holiday feeling that customers associate with cozy, familiar celebrations.
-- Their silhouette and rotation reinforce a seasonal theme, making the piece feel like a refined, gift-worthy decoration.
-- Adds warmth and a ceremonious, festive atmosphere suited for family dinners and elegant gatherings.
-Whimsical walking reindeer
-- Introduces playful, charming motion that lightens the mood and feels more storybook or nostalgic.
-- Creates animated shadow play and a lively centerpiece effect that customers find enchanting for casual or family-focused settings.
-Shared design elements that shape perception
-- Precision-cut, heat-responsive alloy with silver and gold finishes enhances light play and perceived luxury.
-- The overall rotating movement and shadow casting are repeatedly described as mesmerizing, transforming routine candle use into a warm, magical ritual.</t>
+          <t>Short answer: the charm variations (silver snowflakes, standing pine trees, and whimsical reindeer), their high‑shine metal finishes, and the embossed glass all interact with the heat‑driven rotation to change the winter festive atmosphere in distinct ways that customers notice and praise.
+Snowflake charms
+- High‑shine silver snowflakes catch and double the light reflections from the deeply textured, embossed glass.
+- Their rotation casts rhythmic, dancing shadows across walls and mirrors, creating a mesmerizing, dreamlike focal point.
+- Customers describe this combination as elevating a candle ritual into a therapeutic, high‑end holiday moment.
+Standing holiday pine tree charms
+- The pine tree motif reinforces a traditional winter holiday theme, giving a classic, familiar festive atmosphere.
+- Seen as especially suitable for formal holiday centerpieces and luxury gift sets; it strengthens the product’s seasonal, elegant feel.
+Whimsical walking reindeer charms
+- The reindeer add a playful, storybook quality to the motion, contributing a charming, cozy vibe.
+- Their movement enhances the kinetic, mesmerizing effect customers find captivating.
+Metal finishes + embossed glass (overall effect)
+- Precision‑cut alloy in high‑shine silver and polished gold combined with rose‑gold/amber embossed glass amplifies reflections and seasonal warmth.
+- The heat‑powered rotation turns static candle decor into a dynamic, luxurious centerpiece—perceived as dreamy, magical, and festive.
+Bottom line: customers feel each charm variation shifts the mood—from magical and reflective (snowflakes), to traditional and giftable (pine trees), to whimsical and cozy (reindeer)—while the finishes and embossed glass consistently raise the piece’s luxurious, mesmerizing holiday presence.</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1130,7 +1214,10 @@
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>10.12</v>
+        <v>15.5</v>
+      </c>
+      <c r="H16" t="n">
+        <v>9.76</v>
       </c>
     </row>
     <row r="17">
@@ -1146,17 +1233,18 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>### Why the faces are smoothly sanded while the bark edge is kept intact
-Functional reasons
-- Smooth sanding on both faces prevents splinters that could damage delicate linens or scratch sensitive tabletops.
-- A uniformly sanded surface (cut to about **1–1.5 cm** thickness) gives stable foundational support so the slice holds heavy glass candle vessels without warping.
-- As a candle coaster, the sanded surface acts as a heat-resistant protective layer, shielding furniture from thermal stress or cracking.
-Aesthetic reasons
-- Sanding brings out the tightly concentric annual growth rings and the raw, unmanufactured forest look that creates a cozy, rustic vibe.
-- Leaving the organic bark trim preserves a handcrafted, natural edge that modern interiors value for atmosphere and authenticity.
-Durability and workmanship
-- The bark is preserved through meticulous artisanal cutting and the pine faces are smoothly sanded, which keeps the bark from peeling or crumbling while maintaining the rustic edge.
-This balance delivers safe, practical tabletop protection and stability, while keeping the warm, natural appearance that makes the piece attractive in home decor.</t>
+          <t>Why this finish is used
+Natural pine tray slices are sanded on both faces while the rough bark edge is left intact to balance practical utility with a rustic look:
+- Safety and protection  
+  - Smooth faces prevent splinters that could damage delicate linens or scratch tabletops.
+- Aesthetic display  
+  - Sanding brings out the tightly concentric growth rings and the organic circular/oval shape, while the preserved bark retains a raw, handcrafted forest aesthetic.
+- Stability and load-bearing  
+  - Uniform cross-cut thickness (about 1–1.5 cm) and smooth faces give a stable, flat surface that supports heavy glass candle vessels.
+- Durable rustic edge  
+  - Meticulous artisanal cutting preserves the bark so it remains stable and non-crumbling rather than peeling away.
+- Dual-purpose usefulness for candles  
+  - The finished face serves as a heat-resistant protective layer for furniture while the bark edge keeps the warm, rustic atmosphere.</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1169,7 +1257,10 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>7.98</v>
+        <v>8.83</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7.19</v>
       </c>
     </row>
     <row r="18">
@@ -1185,26 +1276,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Flat-top cylindrical cap
-- Shape/function
-  - Compact, flat-top cylindrical silhouette that drops straight down.
-- How it optimizes oxygen deprivation
-  - Fits into narrow, confined wax cups and narrow-necked glass containers so the cap can enclose the wick cleanly.
-  - Its straight, compact geometry prevents striking or disturbing delicate glass edges while sealing off air rapidly.
+          <t>Here’s a clear contrast and analysis of the two head styles and how each optimizes oxygen deprivation for different candle vessels.
+Flat-top cylindrical cap
+- Structure: compact, flat-top cylinder with a streamlined geometric silhouette.
+- How it deprives oxygen: drops directly into the vessel and encloses the wick with a tight, compact fit to cut off airflow.
+- Best vessels/use cases:
+  - Narrow, confined wax votive cups (allows clean insertion without striking or disturbing glass edges).
+  - Narrow-necked glass containers (fits easily into tight openings).
+- Practical benefit: space-efficient and precise for multiple small cups or confined openings.
 Flared vintage bell dome
-- Shape/function
-  - Wide, flared bell-shaped dome with a broader coverage area; often offered with a pivoting head on long rods.
-- How it optimizes oxygen deprivation
-  - The wide flare easily covers the exposed wick from any side angle, cutting off oxygen quickly without disturbing slender tapered candles.
-  - A pivoting bell head can automatically meet the wick flatly on high or awkward displays, improving the seal and making extinguishing easier without climbing up.
-Vessel-by-vessel comparison
-- Narrow-necked jars and confined votive cups
-  - Flat-top cylindrical cap is superior because it can drop straight into the opening and seal the wick without hitting the glass.
-- Tapered dining candles
-  - Flared bell dome excels because its wide, angled profile covers the exposed wick from different approach angles and preserves the slim candle shape.
-- Tall or hard-to-reach placements
-  - A flared bell with a pivoting head offers better angle adjustment to form a flat seal over the wick from a distance.
-In short: the flat-top cylinder is optimized for tight openings and confined glass vessels, while the flared bell dome is optimized for broad coverage of exposed wicks (especially tapered candles) and for angle flexibility on elevated displays.</t>
+- Structure: wide, flared bell-shaped dome (often with a vintage, artistic appearance).
+- How it deprives oxygen: the wide flared shape covers the exposed wick from a range of side angles, quickly cutting off oxygen without disturbing slender wicks.
+- Best vessels/use cases:
+  - Tapered dining-table candles (the flared dome easily covers the wick from any angle).
+  - Tall or hard-to-reach displays when paired with a pivoting head (the head can adjust to meet the wick flatly as the rod is raised).
+- Practical benefit: fast, forgiving coverage for exposed or angled wicks and an old‑world aesthetic.
+Quick choice guide
+- Use a flat-top cylinder for narrow-necked jars and multiple small votives where precise, compact insertion matters.
+- Use a flared bell dome for tapered candles, exposed wicks, or when you need wider, angle‑forgiving coverage (and when style matters).</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1217,7 +1306,10 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>11.38</v>
+        <v>12.51</v>
+      </c>
+      <c r="H18" t="n">
+        <v>11.14</v>
       </c>
     </row>
     <row r="19">
@@ -1233,16 +1325,21 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Why this construction makes the tray a versatile multi-room organizer
-- Durability and appearance
-  - The anti-rust gold alloy frame stays reflective and rust-free in high-humidity spaces, so the tray remains elegant and long‑lasting in bathrooms, vanities, or humid rooms.
-- Surface protection and safety
-  - The metal frame plus mirrored glass base prevents high heat from candle bottoms from transferring to and damaging wood, laminate, or marble surfaces, and it catches hot wax mishaps cleanly—making it safe for tabletops and counters.
-- Practical organization
-  - The heavy-duty reflective mirror glass lets you read labels on the bottoms of small bottles or containers via reflection, speeding up sorting and retrieval when used for cosmetics, oils, or small items.
-- Maintenance and cleanliness
-  - The construction protects counters from moisture rings, rust circles, and oil stains, keeping surfaces cleaner across bedrooms, bathrooms, and living areas.
-Together, the anti-rust gold alloy frame and heavy-duty mirror base combine durability, safety, visual appeal, and practical organization—qualities that let the candle metal tray function well as a multi-room organizer.</t>
+          <t>Short answer
+The anti-rust gold alloy frame plus heavy-duty reflective mirror glass base make the candle metal tray durable, protective, and visually useful—so it works as a multi-room organizer.
+How the construction enables multi-room use
+- Long-term durability in humid spaces  
+  - The anti-rust gold alloy frame resists tarnish and corrosion, so the tray stays elegant and functional in high-humidity restrooms and bathrooms.
+- Surface and thermal protection  
+  - The metal frame and mirrored glass prevent high heat from candle bottoms from transferring to and damaging wood, laminate, or marble tabletops, and the mirror catches hot wax mishaps cleanly.
+- Better display and lighting (bedroom/vanity)  
+  - The crystal-clear reflective mirror base amplifies ambient light and the candle glow, creating a glamorous display on a bedroom vanity or dressing table.
+- Practical organization (cosmetics and small items)  
+  - The heavy-duty reflective glass lets you read labels on the bottoms of dropper bottles and small containers by reflection, making sorting and retrieval faster.
+- Protects surfaces from everyday stains  
+  - The tray guards counters from moisture marks, rust circles from metal canisters, and oil stains from glass droppers, keeping surfaces cleaner across rooms.
+Result
+Together, these features make the tray suitable as a protective, attractive, and functional organizer for bathrooms, vanity/bedroom surfaces, and any tabletop where heat, moisture, or small-item organization are concerns.</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1255,7 +1352,10 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>9.01</v>
+        <v>19.33</v>
+      </c>
+      <c r="H19" t="n">
+        <v>7.55</v>
       </c>
     </row>
     <row r="20">
@@ -1271,39 +1371,29 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thesis
-A premium matchbox with a minimalist "Good Day" slide-box design turns lighting a candle from a mere utility into a therapeutic self‑care ritual by combining visual intention, pleasing tactile interaction, dependable function, and prominent display that together reframe the action as a mindful moment.
-Key points
-- Visual framing and mood  
-  - The clean typography and high‑contrast, minimalist aesthetic create a sophisticated, comforting, and intentional atmosphere.  
-  - That aesthetic cues the user to slow down and treat lighting the candle as a deliberate, calming act rather than a hurried task.
-- Tactile satisfaction and ritual mechanics  
-  - The heavy‑duty slider box and honeycomb friction strike pad provide a satisfying, repeatable physical motion.  
-  - That small, designed interaction (sliding the box, striking a long wooden match) becomes a mini‑ritual that grounds attention.
-- Functional safety and ease  
-  - Elongated wood sticks and extra‑long burn time let users light deep‑wick jars without fumbling or burning fingers, removing friction and anxiety from the act.  
-  - Reliable performance supports a smooth, untroubled experience—essential for something intended to soothe.
-- Display and identity  
-  - Stylish packaging invites keeping the matchbox visible on coffee tables, vanity trays, or bath counters.  
-  - Having it on display signals intentional self‑care and reinforces the habit: the accessory itself becomes part of the calming environment.
-- Perceived value and mindset shift  
-  - As a premium, photogenic accessory (an upgrade from a disposable lighter), it reframes the act as meaningful and worth savoring.  
-  - The result is that a simple flame‑lighting transforms into a small, repeated ceremony that supports relaxation and well‑being.
-Conclusion
-By aligning form, feel, function, and placement, the "Good Day" slide‑box design converts a basic utility into a curated, therapeutic ritual—encouraging presence, reducing friction, and making the moment feel intentionally restorative.</t>
+          <t>Here’s a clear, persuasive argument for why a premium matchbox with a minimalist “Good Day” slide-box design turns ordinary candle lighting into a therapeutic self-care ritual:
+- Visual elevation: The minimalist “Good Day” typography and photogenic slide-box design make the matchbox look like intentional home decor rather than a disposable tool. When an object is attractive and meant to be displayed, interacting with it feels more deliberate and special.
+- Ritual-ready placement: People place these matchboxes on coffee tables, vanity trays, bedside candle vanities, and bath counters. Having the matchbox visible alongside favorite candles creates a consistent visual cue to pause and perform a comforting ritual.
+- Thoughtful materials and function: Elongated, eco-friendly wooden matches with clean-burning, sulfur-free tips and an extra-long burn make lighting candles easier and safer. The practical improvement — reaching deep wicks without burning fingers — removes small annoyances and allows the moment to be calm and focused.
+- Tactile, high-quality packaging: A heavy-duty slider box with a honeycomb-textured striker and high-contrast color options gives satisfying tactile feedback and a sense of craftsmanship. That physical interaction — sliding the box, striking the match — encourages mindfulness and presence.
+- Perceived upgrade and mindset shift: Because users see the matchbox as a premium upgrade from cheap lighters, the act of lighting a candle shifts from mere utility to an intentional, self-care gesture. The overall mood created is minimalist, sophisticated, comforting, intentional, therapeutic, and clean — all qualities that support a restorative ritual.
+Together, these design, material, and placement elements transform a quick, functional task into a small, repeatable ceremony that supports relaxation and intentional living.</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>1</v>
       </c>
       <c r="E20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="b">
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>9.42</v>
+        <v>10.89</v>
+      </c>
+      <c r="H20" t="n">
+        <v>8.210000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -1319,16 +1409,21 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>### Recommended accessory combination
-#### Candle Snuffer
-- Best for extinguishing multi-wick and deep-set jar candles (including tall jars and deep votive cups).
-- Helps prevent soot deposits and accidental wax damage, preserving a pristine wax surface and cleaner indoor air.
-#### Wick Trimmer
-- Keeps wick at proper length to reduce soot and smoking, supporting clean burn and a tidy wax pool.
-- Maintains candle fragrance and appearance over multiple uses.
-#### Candle Tray
-- Protects surfaces from stray wax and heat, preserving the candle’s aesthetic and preventing accidental damage.
-Use all three together and follow proper placement, supervision, wick maintenance, and lighting practices to meet your goal of safely extinguishing deep-set jar candles while keeping wax pristine and indoor air clean.</t>
+          <t>Recommended accessory combination
+Candle Snuffer
+- Best choice for safely extinguishing multi-wick and deep-set jar candles (also works for tall jars, deep votives, tapered candles, and hard-to-reach wicks).
+- Benefit: Lets you put flames out without disturbing the wax surface, helping preserve a pristine appearance.
+Wick Trimmer
+- Use for regular wick maintenance to keep wicks at the proper length before relighting.
+- Benefit: Reduces soot and uneven burning, supporting cleaner indoor air and a neater wax pool.
+Protective Tray
+- Place candles on a high-quality tray to catch any stray wax or drips and protect surfaces.
+- Benefit: Prevents accidental wax damage while keeping the display elegant.
+How to use them together (brief)
+- Trim wicks before lighting.
+- Burn as usual on the tray to protect surfaces.
+- Extinguish with the snuffer to avoid smoke, soot, and wax disruption—maintaining fragrance, ambiance, and a clean appearance.
+This combination best matches your goal of safely extinguishing multiple deep-set jar candles while preserving wax appearance and cleaner indoor air.</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1341,7 +1436,10 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>9</v>
+        <v>15.99</v>
+      </c>
+      <c r="H21" t="n">
+        <v>10.37</v>
       </c>
     </row>
   </sheetData>
@@ -1400,9 +1498,87 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>328</v>
+        <v>499</v>
       </c>
       <c r="E2" t="inlineStr">
+        <is>
+          <t>Question:
+                    Why should users avoid blowing out candles with their breath when a specialized candle snuffer tool is available?
+                    Answer:
+                    Blowing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Formulate a sound structural argument explaining why utilizing a specialized long-handled candle snuffer entirely eliminates the primary hỏa hoạn hazards and odor contamination associated with blowing out candle wicks.</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FAQ_Accesories_product.json</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>461</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Question:
+                    How does using a long-handled candle snuffer protect the fragrance integrity of a room after extinguishing a flame?
+                    Answer:
+                    A can</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Formulate a sound structural argument explaining why utilizing a specialized long-handled candle snuffer entirely eliminates the primary hỏa hoạn hazards and odor contamination associated with blowing out candle wicks.</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FAQ_Accesories_product.json</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>500</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Question:
+                    What structural advantage does an extra-long straight rod handle with an integrated ergonomic grip give to a candle snuffer user?
+                    Answer:
+           </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Formulate a sound structural argument explaining why utilizing a specialized long-handled candle snuffer entirely eliminates the primary hỏa hoạn hazards and odor contamination associated with blowing out candle wicks.</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FAQ_Accesories_product.json</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>468</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t xml:space="preserve">Question:
                     What specific safety risk is completely eliminated when replacing the act of hard blowing with a pivoting-head candle snuffer?
@@ -1411,84 +1587,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Formulate a sound structural argument explaining why utilizing a specialized long-handled candle snuffer entirely eliminates the primary hỏa hoạn hazards and odor contamination associated with blowing out candle wicks.</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>FAQ_Accesories_product.json</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>359</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Question:
-                    Why should users avoid blowing out candles with their breath when a specialized candle snuffer tool is available?
-                    Answer:
-                    Blowing</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Formulate a sound structural argument explaining why utilizing a specialized long-handled candle snuffer entirely eliminates the primary hỏa hoạn hazards and odor contamination associated with blowing out candle wicks.</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>FAQ_Accesories_product.json</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>321</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Question:
-                    How does using a long-handled candle snuffer protect the fragrance integrity of a room after extinguishing a flame?
-                    Answer:
-                    A can</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Formulate a sound structural argument explaining why utilizing a specialized long-handled candle snuffer entirely eliminates the primary hỏa hoạn hazards and odor contamination associated with blowing out candle wicks.</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>FAQ_Accesories_product.json</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>360</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Question:
-                    What structural advantage does an extra-long straight rod handle with an integrated ergonomic grip give to a candle snuffer user?
-                    Answer:
-           </t>
-        </is>
-      </c>
-    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1504,14 +1602,14 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>365</v>
+        <v>515</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Question:
-                    What is the ultimate objective of using specialized candle care tools like scissors and snuffers during a relaxation ritual?
-                    Answer:
-                </t>
+          <t>Question:
+                    How does a textured ergonomic grip at the tail handle of a candle snuffer enhance safe handling?
+                    Answer:
+                    It prevents slippage and</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1628,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>320</v>
+        <v>460</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1556,7 +1654,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>327</v>
+        <v>467</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1582,7 +1680,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>377</v>
+        <v>517</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1608,7 +1706,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>345</v>
+        <v>485</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1634,7 +1732,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>414</v>
+        <v>554</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1660,7 +1758,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>322</v>
+        <v>462</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1686,7 +1784,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>330</v>
+        <v>470</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1712,7 +1810,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>343</v>
+        <v>483</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1738,7 +1836,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>397</v>
+        <v>537</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1764,7 +1862,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>369</v>
+        <v>509</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1790,7 +1888,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>347</v>
+        <v>487</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1816,7 +1914,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>232</v>
+        <v>372</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1838,18 +1936,15 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FAQ_Accesories_product.json</t>
+          <t>FAQ_Product_Catalog.json</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>324</v>
+        <v>148</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Question:
-                    What is the structural utility of the slightly raised rim on a minimalist stainless steel candle tray?
-                    Answer:
-                    The slightly raise</t>
+          <t>What category does Candle metal tray belong to?</t>
         </is>
       </c>
     </row>
@@ -1864,13 +1959,39 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>FAQ_Accesories_product.json</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>464</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Question:
+                    What is the structural utility of the slightly raised rim on a minimalist stainless steel candle tray?
+                    Answer:
+                    The slightly raise</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Compare the material composition, visual design intentions, and specific structural protection features of the minimalist capsule Candle Tray versus the royal gold Candle metal tray.</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>Candle_Tray.md</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>35</v>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="D21" t="n">
+        <v>75</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>Product name: Candle Tray
 Category: Candle Accessory / Organizer Tray / Decorative Plate
@@ -1879,32 +2000,6 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Compare the material composition, visual design intentions, and specific structural protection features of the minimalist capsule Candle Tray versus the royal gold Candle metal tray.</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>5</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>FAQ_Product_Catalog.json</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>214</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Question:
-                    What mood does Candle Tray create?
-                    Answer:
-                    Minimalist, neat, organized, sophisticated, polished.</t>
-        </is>
-      </c>
-    </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -1920,7 +2015,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>339</v>
+        <v>479</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1946,7 +2041,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>386</v>
+        <v>526</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1972,7 +2067,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>418</v>
+        <v>558</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1998,7 +2093,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2024,7 +2119,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>382</v>
+        <v>522</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2050,7 +2145,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>407</v>
+        <v>547</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2076,7 +2171,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>383</v>
+        <v>523</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2102,7 +2197,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>415</v>
+        <v>555</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2128,7 +2223,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>429</v>
+        <v>569</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2154,7 +2249,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>366</v>
+        <v>506</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2180,7 +2275,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>386</v>
+        <v>526</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2206,7 +2301,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2232,7 +2327,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>331</v>
+        <v>471</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2258,7 +2353,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>416</v>
+        <v>556</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2284,7 +2379,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>323</v>
+        <v>463</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2310,7 +2405,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>335</v>
+        <v>475</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2336,7 +2431,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2364,7 +2459,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2390,14 +2485,11 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>217</v>
+        <v>137</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Question:
-                    What are the main scents of Candle holder?
-                    Answer:
-                    - Unspecified - Decorative Product</t>
+          <t>What are the main scents of Candle holder?</t>
         </is>
       </c>
     </row>
@@ -2416,14 +2508,14 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>219</v>
+        <v>357</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>Question:
-                    What fragrance family is Candle holder in?
-                    Answer:
-                    Decorative / Unscented</t>
+                    What are the main scents of Candle holder?
+                    Answer:
+                    - Unspecified - Decorative Product</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2534,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>404</v>
+        <v>544</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2468,7 +2560,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>388</v>
+        <v>528</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2494,7 +2586,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>347</v>
+        <v>487</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2520,7 +2612,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>394</v>
+        <v>534</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2546,7 +2638,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>341</v>
+        <v>481</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2572,7 +2664,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>393</v>
+        <v>533</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2598,7 +2690,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>357</v>
+        <v>497</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2624,7 +2716,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>223</v>
+        <v>363</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2650,7 +2742,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>416</v>
+        <v>556</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2672,18 +2764,15 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FAQ_Accesories_product.json</t>
+          <t>FAQ_Product_Catalog.json</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>371</v>
+        <v>143</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Question:
-                    What is the primary formulation difference between premium safety matches and cheap standard utility matchboxes?
-                    Answer:
-                    Premium </t>
+          <t>What are the main scents of Candle matchbox?</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2791,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>356</v>
+        <v>496</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2728,7 +2817,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>332</v>
+        <v>472</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2754,7 +2843,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>337</v>
+        <v>477</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2780,7 +2869,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>401</v>
+        <v>541</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2806,7 +2895,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>324</v>
+        <v>464</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2832,7 +2921,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>431</v>
+        <v>571</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2858,7 +2947,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>309</v>
+        <v>449</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -2884,7 +2973,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>320</v>
+        <v>460</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2910,7 +2999,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>354</v>
+        <v>494</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2936,7 +3025,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>399</v>
+        <v>539</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2962,7 +3051,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>415</v>
+        <v>555</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -2988,7 +3077,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>395</v>
+        <v>535</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -3014,7 +3103,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>355</v>
+        <v>495</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -3040,7 +3129,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>342</v>
+        <v>482</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3066,7 +3155,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3091,7 +3180,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>402</v>
+        <v>542</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3117,7 +3206,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3143,7 +3232,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>559</v>
+        <v>699</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3169,7 +3258,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3195,7 +3284,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>59</v>
+        <v>99</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3221,7 +3310,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>330</v>
+        <v>470</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3247,7 +3336,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>400</v>
+        <v>540</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -3273,7 +3362,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3298,7 +3387,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>348</v>
+        <v>488</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3324,7 +3413,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>238</v>
+        <v>378</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -3350,7 +3439,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>344</v>
+        <v>484</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -3376,7 +3465,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>364</v>
+        <v>504</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3402,7 +3491,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>410</v>
+        <v>550</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -3428,7 +3517,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>333</v>
+        <v>473</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -3454,7 +3543,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>326</v>
+        <v>466</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -3480,7 +3569,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>334</v>
+        <v>474</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -3506,7 +3595,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>387</v>
+        <v>527</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -3532,7 +3621,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>362</v>
+        <v>502</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -3558,7 +3647,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>411</v>
+        <v>551</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -3584,7 +3673,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>372</v>
+        <v>512</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -3610,7 +3699,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>379</v>
+        <v>519</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -3636,7 +3725,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>342</v>
+        <v>482</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -3662,7 +3751,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>325</v>
+        <v>465</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -3688,7 +3777,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>401</v>
+        <v>541</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -3714,7 +3803,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>398</v>
+        <v>538</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3740,7 +3829,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>386</v>
+        <v>526</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -3766,7 +3855,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>226</v>
+        <v>366</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -3788,13 +3877,36 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
+          <t>FAQ_Product_Catalog.json</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>146</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>What mood does Candle matchbox create?</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Formulate an argument explaining why a premium candle matchbox featuring an aesthetic 'Good Day' slide-box design transforms a basic utility act into a therapeutic self-care ritual.</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>4</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
           <t>Candle_matchbox.md</t>
         </is>
       </c>
-      <c r="D94" t="n">
-        <v>29</v>
-      </c>
-      <c r="E94" t="inlineStr">
+      <c r="D95" t="n">
+        <v>69</v>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>Product name: Candle matchbox
 Category: Candle Accessory / Luxury Safety Matches
@@ -3803,32 +3915,6 @@
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Formulate an argument explaining why a premium candle matchbox featuring an aesthetic 'Good Day' slide-box design transforms a basic utility act into a therapeutic self-care ritual.</t>
-        </is>
-      </c>
-      <c r="B95" t="n">
-        <v>4</v>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>FAQ_Accesories_product.json</t>
-        </is>
-      </c>
-      <c r="D95" t="n">
-        <v>407</v>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Question:
-                    Why is the premium rose-gold or amber glass container of a luxury candle often designed with a deeply textured pattern?
-                    Answer:
-                    T</t>
-        </is>
-      </c>
-    </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
@@ -3844,14 +3930,14 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>374</v>
+        <v>547</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>Question:
-                    What specific consumer group or demographic is a white slide-box match box with snow-white tips designed to attract?
-                    Answer:
-                    Cons</t>
+                    Why is the premium rose-gold or amber glass container of a luxury candle often designed with a deeply textured pattern?
+                    Answer:
+                    T</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3956,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>418</v>
+        <v>558</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3896,7 +3982,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>317</v>
+        <v>457</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3922,7 +4008,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>209</v>
+        <v>349</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3948,7 +4034,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>518</v>
+        <v>658</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -3974,7 +4060,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>299</v>
+        <v>439</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>

</xml_diff>